<commit_message>
Do not leave unused formats in the stylesheet under a global style
</commit_message>
<xml_diff>
--- a/src/Excelsior.Tests/StyleTests.GlobalStyle.verified.xlsx
+++ b/src/Excelsior.Tests/StyleTests.GlobalStyle.verified.xlsx
@@ -12,13 +12,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-MM-dd"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
@@ -51,20 +46,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0"/>
-    <xf fontId="1" fillId="0" borderId="0" applyFont="1" applyFill="0"/>
-    <xf fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyAlignment="1">
+    <xf fontId="1" fillId="2" borderId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="1" fillId="2" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFont="0" applyFill="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="2" borderId="0" applyFont="1" applyFill="1"/>
-    <xf fontId="2" fillId="2" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -93,153 +81,153 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Employee ID</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Full Name</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Email Address</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Hire Date</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Annual Salary</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Is Active</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5">
-        <v>1</v>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">John Doe</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">john@company.com</t>
         </is>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="3">
         <v>43845</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="2">
         <v>75000</v>
       </c>
-      <c r="F2" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="F2" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Full Time</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Jane Smith</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">jane@company.com</t>
         </is>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="3">
         <v>43546</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="2">
         <v>120000</v>
       </c>
-      <c r="F3" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="F3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Full Time</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Bob Johnson</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">bob@company.com</t>
         </is>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="3">
         <v>44387</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="2">
         <v>45000</v>
       </c>
-      <c r="F4" s="5" t="b">
+      <c r="F4" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Part Time</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Alice Brown</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">alice@company.com</t>
         </is>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="3">
         <v>43409</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="2">
         <v>95000</v>
       </c>
-      <c r="F5" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Contract</t>
         </is>

</xml_diff>

<commit_message>
Measure column widths and apply the global style as cells are written
</commit_message>
<xml_diff>
--- a/src/Excelsior.Tests/StyleTests.GlobalStyle.verified.xlsx
+++ b/src/Excelsior.Tests/StyleTests.GlobalStyle.verified.xlsx
@@ -12,13 +12,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-MM-dd"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
@@ -51,20 +46,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0"/>
-    <xf fontId="1" fillId="0" borderId="0" applyFont="1" applyFill="0"/>
-    <xf fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyAlignment="1">
+    <xf fontId="1" fillId="2" borderId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="1" fillId="2" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFont="0" applyFill="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="2" borderId="0" applyFont="1" applyFill="1"/>
-    <xf fontId="2" fillId="2" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -93,153 +81,153 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Employee ID</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Full Name</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Email Address</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Hire Date</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Annual Salary</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Is Active</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5">
-        <v>1</v>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">John Doe</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">john@company.com</t>
         </is>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="3">
         <v>43845</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="2">
         <v>75000</v>
       </c>
-      <c r="F2" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="F2" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Full Time</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Jane Smith</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">jane@company.com</t>
         </is>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="3">
         <v>43546</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="2">
         <v>120000</v>
       </c>
-      <c r="F3" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="F3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Full Time</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Bob Johnson</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">bob@company.com</t>
         </is>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="3">
         <v>44387</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="2">
         <v>45000</v>
       </c>
-      <c r="F4" s="5" t="b">
+      <c r="F4" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Part Time</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Alice Brown</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">alice@company.com</t>
         </is>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="3">
         <v>43409</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="2">
         <v>95000</v>
       </c>
-      <c r="F5" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Contract</t>
         </is>

</xml_diff>

<commit_message>
Do not leave unused formats in the stylesheet under a global style (#280)
</commit_message>
<xml_diff>
--- a/src/Excelsior.Tests/StyleTests.GlobalStyle.verified.xlsx
+++ b/src/Excelsior.Tests/StyleTests.GlobalStyle.verified.xlsx
@@ -12,13 +12,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-MM-dd"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
@@ -51,20 +46,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0"/>
-    <xf fontId="1" fillId="0" borderId="0" applyFont="1" applyFill="0"/>
-    <xf fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyAlignment="1">
+    <xf fontId="1" fillId="2" borderId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="1" fillId="2" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFont="0" applyFill="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="2" fillId="2" borderId="0" applyFont="1" applyFill="1"/>
-    <xf fontId="2" fillId="2" borderId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -93,153 +81,153 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Employee ID</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Full Name</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Email Address</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Hire Date</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Annual Salary</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Is Active</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5">
-        <v>1</v>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">John Doe</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">john@company.com</t>
         </is>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="3">
         <v>43845</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="2">
         <v>75000</v>
       </c>
-      <c r="F2" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="F2" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Full Time</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Jane Smith</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">jane@company.com</t>
         </is>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="3">
         <v>43546</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="2">
         <v>120000</v>
       </c>
-      <c r="F3" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="F3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Full Time</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Bob Johnson</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">bob@company.com</t>
         </is>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="3">
         <v>44387</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="2">
         <v>45000</v>
       </c>
-      <c r="F4" s="5" t="b">
+      <c r="F4" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Part Time</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Alice Brown</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">alice@company.com</t>
         </is>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="3">
         <v>43409</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="2">
         <v>95000</v>
       </c>
-      <c r="F5" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Contract</t>
         </is>

</xml_diff>